<commit_message>
UPL Addition of missing club data
</commit_message>
<xml_diff>
--- a/Catapult Match Report_FWSL.xlsx
+++ b/Catapult Match Report_FWSL.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnyanzi\Desktop\FUFA\Match-Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e184d086cb18a9d7/Desktop/FUFA/Match_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83EE0A3C-5BB3-4A2D-B9A9-6CE7D77ED267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{83EE0A3C-5BB3-4A2D-B9A9-6CE7D77ED267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D16CA787-46A1-449D-8906-EC5FFF383166}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Club Name</t>
   </si>
@@ -73,13 +74,130 @@
   </si>
   <si>
     <t>Rines SS WFC</t>
+  </si>
+  <si>
+    <t>MD1</t>
+  </si>
+  <si>
+    <t>MD2</t>
+  </si>
+  <si>
+    <t>MD3</t>
+  </si>
+  <si>
+    <t>MD4</t>
+  </si>
+  <si>
+    <t>MD5</t>
+  </si>
+  <si>
+    <t>MD6</t>
+  </si>
+  <si>
+    <t>MD7</t>
+  </si>
+  <si>
+    <t>MD8</t>
+  </si>
+  <si>
+    <t>MD9</t>
+  </si>
+  <si>
+    <t>MD10</t>
+  </si>
+  <si>
+    <t>MD11</t>
+  </si>
+  <si>
+    <t>MD12</t>
+  </si>
+  <si>
+    <t>MD13</t>
+  </si>
+  <si>
+    <t>MD14</t>
+  </si>
+  <si>
+    <t>MD15</t>
+  </si>
+  <si>
+    <t>MD16</t>
+  </si>
+  <si>
+    <t>MD17</t>
+  </si>
+  <si>
+    <t>MD18</t>
+  </si>
+  <si>
+    <t>MD19</t>
+  </si>
+  <si>
+    <t>MD20</t>
+  </si>
+  <si>
+    <t>MD21</t>
+  </si>
+  <si>
+    <t>MD22</t>
+  </si>
+  <si>
+    <t>Match Day</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>Sprint Distance</t>
+  </si>
+  <si>
+    <t>Power Plays</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Impacts</t>
+  </si>
+  <si>
+    <t>Total Accelerations</t>
+  </si>
+  <si>
+    <t>Total Decelerations</t>
+  </si>
+  <si>
+    <t>Player Load</t>
+  </si>
+  <si>
+    <t>Top Speed</t>
+  </si>
+  <si>
+    <t>Distance Per Minute</t>
+  </si>
+  <si>
+    <t>Power Score</t>
+  </si>
+  <si>
+    <t>Work Ratio</t>
+  </si>
+  <si>
+    <t>Max Acceleration</t>
+  </si>
+  <si>
+    <t>Max Deceleration</t>
+  </si>
+  <si>
+    <t>Accelerations Per Minute</t>
+  </si>
+  <si>
+    <t>Decelerations Per Minute</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +215,25 @@
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -142,12 +279,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -215,8 +364,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.11220285150722401"/>
-          <c:y val="1.8518518518518517E-2"/>
+          <c:x val="0.10665500210701787"/>
+          <c:y val="5.4109528443775916E-4"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1154,16 +1303,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>142874</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>390524</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>15875</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1455,14 +1604,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.1796875" customWidth="1"/>
-    <col min="3" max="3" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:3" ht="23.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1470,7 +1619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1478,7 +1627,7 @@
         <v>12.052631999999999</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1486,7 +1635,7 @@
         <v>11.571429</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
@@ -1494,7 +1643,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1502,7 +1651,7 @@
         <v>11.105263000000001</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1510,7 +1659,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="23.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:3" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
@@ -1518,7 +1667,7 @@
         <v>10.411765000000001</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
@@ -1526,7 +1675,7 @@
         <v>10.294117999999999</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1534,7 +1683,7 @@
         <v>9.4545449999999995</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1542,7 +1691,7 @@
         <v>7.2727269999999997</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1550,7 +1699,7 @@
         <v>6.6666670000000003</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1565,4 +1714,1439 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D5576CA-012C-40B7-A563-0EDE6BB4AF59}">
+  <dimension ref="B1:R24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="7.5703125" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="14" width="7.7109375" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" customWidth="1"/>
+    <col min="16" max="16" width="10" customWidth="1"/>
+    <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="18" max="18" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="6">
+        <v>6.96</v>
+      </c>
+      <c r="D3" s="6">
+        <v>348.88</v>
+      </c>
+      <c r="E3" s="6">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="F3" s="6">
+        <v>687.38</v>
+      </c>
+      <c r="G3" s="6">
+        <v>5.58</v>
+      </c>
+      <c r="H3" s="6">
+        <v>346.91</v>
+      </c>
+      <c r="I3" s="6">
+        <v>335.01</v>
+      </c>
+      <c r="J3" s="6">
+        <v>343.95</v>
+      </c>
+      <c r="K3" s="6">
+        <v>25.13</v>
+      </c>
+      <c r="L3" s="6">
+        <v>71.05</v>
+      </c>
+      <c r="M3" s="6">
+        <v>11.01</v>
+      </c>
+      <c r="N3" s="6">
+        <v>56.85</v>
+      </c>
+      <c r="O3" s="6">
+        <v>5.12</v>
+      </c>
+      <c r="P3" s="6">
+        <v>6.15</v>
+      </c>
+      <c r="Q3" s="6">
+        <v>3.54</v>
+      </c>
+      <c r="R3" s="6">
+        <v>3.42</v>
+      </c>
+    </row>
+    <row r="4" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="6">
+        <v>7.1</v>
+      </c>
+      <c r="D4" s="6">
+        <v>392.41</v>
+      </c>
+      <c r="E4" s="6">
+        <v>34.89</v>
+      </c>
+      <c r="F4" s="6">
+        <v>699.78</v>
+      </c>
+      <c r="G4" s="6">
+        <v>5.38</v>
+      </c>
+      <c r="H4" s="6">
+        <v>346.81</v>
+      </c>
+      <c r="I4" s="6">
+        <v>335.23</v>
+      </c>
+      <c r="J4" s="6">
+        <v>352.28</v>
+      </c>
+      <c r="K4" s="6">
+        <v>25.41</v>
+      </c>
+      <c r="L4" s="6">
+        <v>68.98</v>
+      </c>
+      <c r="M4" s="6">
+        <v>10.73</v>
+      </c>
+      <c r="N4" s="6">
+        <v>54.96</v>
+      </c>
+      <c r="O4" s="6">
+        <v>5.15</v>
+      </c>
+      <c r="P4" s="6">
+        <v>6.42</v>
+      </c>
+      <c r="Q4" s="6">
+        <v>3.38</v>
+      </c>
+      <c r="R4" s="6">
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="6">
+        <v>7.37</v>
+      </c>
+      <c r="D5" s="6">
+        <v>440.24</v>
+      </c>
+      <c r="E5" s="6">
+        <v>40.4</v>
+      </c>
+      <c r="F5" s="6">
+        <v>738.66</v>
+      </c>
+      <c r="G5" s="6">
+        <v>6.65</v>
+      </c>
+      <c r="H5" s="6">
+        <v>364.79</v>
+      </c>
+      <c r="I5" s="6">
+        <v>355.85</v>
+      </c>
+      <c r="J5" s="6">
+        <v>364.28</v>
+      </c>
+      <c r="K5" s="6">
+        <v>25.44</v>
+      </c>
+      <c r="L5" s="6">
+        <v>76.180000000000007</v>
+      </c>
+      <c r="M5" s="6">
+        <v>11.79</v>
+      </c>
+      <c r="N5" s="6">
+        <v>60.94</v>
+      </c>
+      <c r="O5" s="6">
+        <v>5.28</v>
+      </c>
+      <c r="P5" s="6">
+        <v>6.52</v>
+      </c>
+      <c r="Q5" s="6">
+        <v>3.77</v>
+      </c>
+      <c r="R5" s="6">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="6">
+        <v>7.26</v>
+      </c>
+      <c r="D6" s="6">
+        <v>429.24</v>
+      </c>
+      <c r="E6" s="6">
+        <v>36.58</v>
+      </c>
+      <c r="F6" s="6">
+        <v>716.33</v>
+      </c>
+      <c r="G6" s="6">
+        <v>5.68</v>
+      </c>
+      <c r="H6" s="6">
+        <v>346.61</v>
+      </c>
+      <c r="I6" s="6">
+        <v>337.69</v>
+      </c>
+      <c r="J6" s="6">
+        <v>351.87</v>
+      </c>
+      <c r="K6" s="6">
+        <v>25.52</v>
+      </c>
+      <c r="L6" s="6">
+        <v>74.069999999999993</v>
+      </c>
+      <c r="M6" s="6">
+        <v>11.5</v>
+      </c>
+      <c r="N6" s="6">
+        <v>59.14</v>
+      </c>
+      <c r="O6" s="6">
+        <v>5.28</v>
+      </c>
+      <c r="P6" s="6">
+        <v>6.51</v>
+      </c>
+      <c r="Q6" s="6">
+        <v>3.54</v>
+      </c>
+      <c r="R6" s="6">
+        <v>3.45</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="6">
+        <v>7.27</v>
+      </c>
+      <c r="D7" s="6">
+        <v>411.03</v>
+      </c>
+      <c r="E7" s="6">
+        <v>37.659999999999997</v>
+      </c>
+      <c r="F7" s="6">
+        <v>719.44</v>
+      </c>
+      <c r="G7" s="6">
+        <v>6.08</v>
+      </c>
+      <c r="H7" s="6">
+        <v>360.75</v>
+      </c>
+      <c r="I7" s="6">
+        <v>349.19</v>
+      </c>
+      <c r="J7" s="6">
+        <v>359.03</v>
+      </c>
+      <c r="K7" s="6">
+        <v>25.68</v>
+      </c>
+      <c r="L7" s="6">
+        <v>73.03</v>
+      </c>
+      <c r="M7" s="6">
+        <v>11.24</v>
+      </c>
+      <c r="N7" s="6">
+        <v>56.81</v>
+      </c>
+      <c r="O7" s="6">
+        <v>5.55</v>
+      </c>
+      <c r="P7" s="6">
+        <v>6.43</v>
+      </c>
+      <c r="Q7" s="6">
+        <v>3.62</v>
+      </c>
+      <c r="R7" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6">
+        <v>7.1</v>
+      </c>
+      <c r="D8" s="6">
+        <v>395.57</v>
+      </c>
+      <c r="E8" s="6">
+        <v>35.94</v>
+      </c>
+      <c r="F8" s="6">
+        <v>699.52</v>
+      </c>
+      <c r="G8" s="6">
+        <v>4.07</v>
+      </c>
+      <c r="H8" s="6">
+        <v>340.93</v>
+      </c>
+      <c r="I8" s="6">
+        <v>328.38</v>
+      </c>
+      <c r="J8" s="6">
+        <v>342.88</v>
+      </c>
+      <c r="K8" s="6">
+        <v>25.42</v>
+      </c>
+      <c r="L8" s="6">
+        <v>72.89</v>
+      </c>
+      <c r="M8" s="6">
+        <v>11.29</v>
+      </c>
+      <c r="N8" s="6">
+        <v>58.04</v>
+      </c>
+      <c r="O8" s="6">
+        <v>5.14</v>
+      </c>
+      <c r="P8" s="6">
+        <v>6.29</v>
+      </c>
+      <c r="Q8" s="6">
+        <v>3.5</v>
+      </c>
+      <c r="R8" s="6">
+        <v>3.37</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="6">
+        <v>7.47</v>
+      </c>
+      <c r="D9" s="6">
+        <v>430.71</v>
+      </c>
+      <c r="E9" s="6">
+        <v>37.409999999999997</v>
+      </c>
+      <c r="F9" s="6">
+        <v>731.98</v>
+      </c>
+      <c r="G9" s="6">
+        <v>6.19</v>
+      </c>
+      <c r="H9" s="6">
+        <v>358.62</v>
+      </c>
+      <c r="I9" s="6">
+        <v>346.77</v>
+      </c>
+      <c r="J9" s="6">
+        <v>362.86</v>
+      </c>
+      <c r="K9" s="6">
+        <v>25.69</v>
+      </c>
+      <c r="L9" s="6">
+        <v>75.92</v>
+      </c>
+      <c r="M9" s="6">
+        <v>11.73</v>
+      </c>
+      <c r="N9" s="6">
+        <v>59.63</v>
+      </c>
+      <c r="O9" s="6">
+        <v>5.23</v>
+      </c>
+      <c r="P9" s="6">
+        <v>6.5</v>
+      </c>
+      <c r="Q9" s="6">
+        <v>3.65</v>
+      </c>
+      <c r="R9" s="6">
+        <v>3.53</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="6">
+        <v>7.43</v>
+      </c>
+      <c r="D10" s="6">
+        <v>411.87</v>
+      </c>
+      <c r="E10" s="6">
+        <v>37.619999999999997</v>
+      </c>
+      <c r="F10" s="6">
+        <v>727.38</v>
+      </c>
+      <c r="G10" s="6">
+        <v>5.05</v>
+      </c>
+      <c r="H10" s="6">
+        <v>371.06</v>
+      </c>
+      <c r="I10" s="6">
+        <v>361.74</v>
+      </c>
+      <c r="J10" s="6">
+        <v>367.03</v>
+      </c>
+      <c r="K10" s="6">
+        <v>25.08</v>
+      </c>
+      <c r="L10" s="6">
+        <v>75.59</v>
+      </c>
+      <c r="M10" s="6">
+        <v>11.78</v>
+      </c>
+      <c r="N10" s="6">
+        <v>60.59</v>
+      </c>
+      <c r="O10" s="6">
+        <v>4.96</v>
+      </c>
+      <c r="P10" s="6">
+        <v>6.18</v>
+      </c>
+      <c r="Q10" s="6">
+        <v>3.77</v>
+      </c>
+      <c r="R10" s="6">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="6">
+        <v>7.23</v>
+      </c>
+      <c r="D11" s="6">
+        <v>436.33</v>
+      </c>
+      <c r="E11" s="6">
+        <v>38.22</v>
+      </c>
+      <c r="F11" s="6">
+        <v>725.83</v>
+      </c>
+      <c r="G11" s="6">
+        <v>5.34</v>
+      </c>
+      <c r="H11" s="6">
+        <v>337.72</v>
+      </c>
+      <c r="I11" s="6">
+        <v>329.12</v>
+      </c>
+      <c r="J11" s="6">
+        <v>342.34</v>
+      </c>
+      <c r="K11" s="6">
+        <v>25.94</v>
+      </c>
+      <c r="L11" s="6">
+        <v>76.86</v>
+      </c>
+      <c r="M11" s="6">
+        <v>11.91</v>
+      </c>
+      <c r="N11" s="6">
+        <v>60.89</v>
+      </c>
+      <c r="O11" s="6">
+        <v>5.16</v>
+      </c>
+      <c r="P11" s="6">
+        <v>6.6</v>
+      </c>
+      <c r="Q11" s="6">
+        <v>3.59</v>
+      </c>
+      <c r="R11" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="6">
+        <v>7.39</v>
+      </c>
+      <c r="D12" s="6">
+        <v>395</v>
+      </c>
+      <c r="E12" s="6">
+        <v>35.590000000000003</v>
+      </c>
+      <c r="F12" s="6">
+        <v>729.5</v>
+      </c>
+      <c r="G12" s="6">
+        <v>5.33</v>
+      </c>
+      <c r="H12" s="6">
+        <v>352.13</v>
+      </c>
+      <c r="I12" s="6">
+        <v>342.89</v>
+      </c>
+      <c r="J12" s="6">
+        <v>355.18</v>
+      </c>
+      <c r="K12" s="6">
+        <v>25.45</v>
+      </c>
+      <c r="L12" s="6">
+        <v>74.010000000000005</v>
+      </c>
+      <c r="M12" s="6">
+        <v>11.46</v>
+      </c>
+      <c r="N12" s="6">
+        <v>58.13</v>
+      </c>
+      <c r="O12" s="6">
+        <v>5.2</v>
+      </c>
+      <c r="P12" s="6">
+        <v>6.48</v>
+      </c>
+      <c r="Q12" s="6">
+        <v>3.52</v>
+      </c>
+      <c r="R12" s="6">
+        <v>3.43</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="6">
+        <v>7.59</v>
+      </c>
+      <c r="D13" s="6">
+        <v>434.32</v>
+      </c>
+      <c r="E13" s="6">
+        <v>37.21</v>
+      </c>
+      <c r="F13" s="6">
+        <v>747.13</v>
+      </c>
+      <c r="G13" s="6">
+        <v>5.05</v>
+      </c>
+      <c r="H13" s="6">
+        <v>345.22</v>
+      </c>
+      <c r="I13" s="6">
+        <v>335.18</v>
+      </c>
+      <c r="J13" s="6">
+        <v>361.34</v>
+      </c>
+      <c r="K13" s="6">
+        <v>25.69</v>
+      </c>
+      <c r="L13" s="6">
+        <v>76.459999999999994</v>
+      </c>
+      <c r="M13" s="6">
+        <v>11.84</v>
+      </c>
+      <c r="N13" s="6">
+        <v>60.23</v>
+      </c>
+      <c r="O13" s="6">
+        <v>5.24</v>
+      </c>
+      <c r="P13" s="6">
+        <v>6.39</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>3.48</v>
+      </c>
+      <c r="R13" s="6">
+        <v>3.38</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="6">
+        <v>7.65</v>
+      </c>
+      <c r="D14" s="6">
+        <v>462.18</v>
+      </c>
+      <c r="E14" s="6">
+        <v>40.479999999999997</v>
+      </c>
+      <c r="F14" s="6">
+        <v>756.97</v>
+      </c>
+      <c r="G14" s="6">
+        <v>5.76</v>
+      </c>
+      <c r="H14" s="6">
+        <v>372.38</v>
+      </c>
+      <c r="I14" s="6">
+        <v>361.36</v>
+      </c>
+      <c r="J14" s="6">
+        <v>377.9</v>
+      </c>
+      <c r="K14" s="6">
+        <v>25.62</v>
+      </c>
+      <c r="L14" s="6">
+        <v>75.290000000000006</v>
+      </c>
+      <c r="M14" s="6">
+        <v>11.73</v>
+      </c>
+      <c r="N14" s="6">
+        <v>60.03</v>
+      </c>
+      <c r="O14" s="6">
+        <v>5.14</v>
+      </c>
+      <c r="P14" s="6">
+        <v>6.52</v>
+      </c>
+      <c r="Q14" s="6">
+        <v>3.67</v>
+      </c>
+      <c r="R14" s="6">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="6">
+        <v>7.77</v>
+      </c>
+      <c r="D15" s="6">
+        <v>461.14</v>
+      </c>
+      <c r="E15" s="6">
+        <v>39.630000000000003</v>
+      </c>
+      <c r="F15" s="6">
+        <v>763.15</v>
+      </c>
+      <c r="G15" s="6">
+        <v>6.36</v>
+      </c>
+      <c r="H15" s="6">
+        <v>354.46</v>
+      </c>
+      <c r="I15" s="6">
+        <v>343.89</v>
+      </c>
+      <c r="J15" s="6">
+        <v>376.81</v>
+      </c>
+      <c r="K15" s="6">
+        <v>25.73</v>
+      </c>
+      <c r="L15" s="6">
+        <v>77.14</v>
+      </c>
+      <c r="M15" s="6">
+        <v>11.96</v>
+      </c>
+      <c r="N15" s="6">
+        <v>61.43</v>
+      </c>
+      <c r="O15" s="6">
+        <v>5.19</v>
+      </c>
+      <c r="P15" s="6">
+        <v>6.41</v>
+      </c>
+      <c r="Q15" s="6">
+        <v>3.53</v>
+      </c>
+      <c r="R15" s="6">
+        <v>3.42</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="6">
+        <v>7.33</v>
+      </c>
+      <c r="D16" s="6">
+        <v>402.64</v>
+      </c>
+      <c r="E16" s="6">
+        <v>34.99</v>
+      </c>
+      <c r="F16" s="6">
+        <v>692.36</v>
+      </c>
+      <c r="G16" s="6">
+        <v>5.6</v>
+      </c>
+      <c r="H16" s="6">
+        <v>343.69</v>
+      </c>
+      <c r="I16" s="6">
+        <v>333.92</v>
+      </c>
+      <c r="J16" s="6">
+        <v>361.38</v>
+      </c>
+      <c r="K16" s="6">
+        <v>25.66</v>
+      </c>
+      <c r="L16" s="6">
+        <v>74.540000000000006</v>
+      </c>
+      <c r="M16" s="6">
+        <v>11.5</v>
+      </c>
+      <c r="N16" s="6">
+        <v>58.69</v>
+      </c>
+      <c r="O16" s="6">
+        <v>5.25</v>
+      </c>
+      <c r="P16" s="6">
+        <v>6.47</v>
+      </c>
+      <c r="Q16" s="6">
+        <v>3.5</v>
+      </c>
+      <c r="R16" s="6">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="6">
+        <v>7.72</v>
+      </c>
+      <c r="D17" s="6">
+        <v>504.49</v>
+      </c>
+      <c r="E17" s="6">
+        <v>42.44</v>
+      </c>
+      <c r="F17" s="6">
+        <v>753.95</v>
+      </c>
+      <c r="G17" s="6">
+        <v>6.58</v>
+      </c>
+      <c r="H17" s="6">
+        <v>349.56</v>
+      </c>
+      <c r="I17" s="6">
+        <v>338</v>
+      </c>
+      <c r="J17" s="6">
+        <v>371.56</v>
+      </c>
+      <c r="K17" s="6">
+        <v>26.13</v>
+      </c>
+      <c r="L17" s="6">
+        <v>80.05</v>
+      </c>
+      <c r="M17" s="6">
+        <v>12.42</v>
+      </c>
+      <c r="N17" s="6">
+        <v>62.67</v>
+      </c>
+      <c r="O17" s="6">
+        <v>5.32</v>
+      </c>
+      <c r="P17" s="6">
+        <v>6.73</v>
+      </c>
+      <c r="Q17" s="6">
+        <v>3.62</v>
+      </c>
+      <c r="R17" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="6">
+        <v>7.3</v>
+      </c>
+      <c r="D18" s="6">
+        <v>408.98</v>
+      </c>
+      <c r="E18" s="6">
+        <v>35.979999999999997</v>
+      </c>
+      <c r="F18" s="6">
+        <v>725.6</v>
+      </c>
+      <c r="G18" s="6">
+        <v>6.4</v>
+      </c>
+      <c r="H18" s="6">
+        <v>348.46</v>
+      </c>
+      <c r="I18" s="6">
+        <v>337.96</v>
+      </c>
+      <c r="J18" s="6">
+        <v>359.75</v>
+      </c>
+      <c r="K18" s="6">
+        <v>25.62</v>
+      </c>
+      <c r="L18" s="6">
+        <v>73.23</v>
+      </c>
+      <c r="M18" s="6">
+        <v>11.35</v>
+      </c>
+      <c r="N18" s="6">
+        <v>57.52</v>
+      </c>
+      <c r="O18" s="6">
+        <v>5.24</v>
+      </c>
+      <c r="P18" s="6">
+        <v>6.33</v>
+      </c>
+      <c r="Q18" s="6">
+        <v>3.5</v>
+      </c>
+      <c r="R18" s="6">
+        <v>3.39</v>
+      </c>
+    </row>
+    <row r="19" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="6">
+        <v>7.3</v>
+      </c>
+      <c r="D19" s="6">
+        <v>427.87</v>
+      </c>
+      <c r="E19" s="6">
+        <v>37.590000000000003</v>
+      </c>
+      <c r="F19" s="6">
+        <v>720.39</v>
+      </c>
+      <c r="G19" s="6">
+        <v>6.68</v>
+      </c>
+      <c r="H19" s="6">
+        <v>351.06</v>
+      </c>
+      <c r="I19" s="6">
+        <v>345.73</v>
+      </c>
+      <c r="J19" s="6">
+        <v>363.08</v>
+      </c>
+      <c r="K19" s="6">
+        <v>25.28</v>
+      </c>
+      <c r="L19" s="6">
+        <v>72.040000000000006</v>
+      </c>
+      <c r="M19" s="6">
+        <v>11.2</v>
+      </c>
+      <c r="N19" s="6">
+        <v>56.71</v>
+      </c>
+      <c r="O19" s="6">
+        <v>5.2</v>
+      </c>
+      <c r="P19" s="6">
+        <v>6.31</v>
+      </c>
+      <c r="Q19" s="6">
+        <v>3.46</v>
+      </c>
+      <c r="R19" s="6">
+        <v>3.41</v>
+      </c>
+    </row>
+    <row r="20" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="6">
+        <v>7.51</v>
+      </c>
+      <c r="D20" s="6">
+        <v>410.82</v>
+      </c>
+      <c r="E20" s="6">
+        <v>38.22</v>
+      </c>
+      <c r="F20" s="6">
+        <v>750.04</v>
+      </c>
+      <c r="G20" s="6">
+        <v>5.33</v>
+      </c>
+      <c r="H20" s="6">
+        <v>372.11</v>
+      </c>
+      <c r="I20" s="6">
+        <v>360.75</v>
+      </c>
+      <c r="J20" s="6">
+        <v>385.48</v>
+      </c>
+      <c r="K20" s="6">
+        <v>25.69</v>
+      </c>
+      <c r="L20" s="6">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="M20" s="6">
+        <v>12.14</v>
+      </c>
+      <c r="N20" s="6">
+        <v>61.43</v>
+      </c>
+      <c r="O20" s="6">
+        <v>5.18</v>
+      </c>
+      <c r="P20" s="6">
+        <v>6.64</v>
+      </c>
+      <c r="Q20" s="6">
+        <v>3.86</v>
+      </c>
+      <c r="R20" s="6">
+        <v>3.74</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="6">
+        <v>7.14</v>
+      </c>
+      <c r="D21" s="6">
+        <v>470.72</v>
+      </c>
+      <c r="E21" s="6">
+        <v>38.979999999999997</v>
+      </c>
+      <c r="F21" s="6">
+        <v>719.56</v>
+      </c>
+      <c r="G21" s="6">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="H21" s="6">
+        <v>335.31</v>
+      </c>
+      <c r="I21" s="6">
+        <v>323.29000000000002</v>
+      </c>
+      <c r="J21" s="6">
+        <v>347.77</v>
+      </c>
+      <c r="K21" s="6">
+        <v>26.28</v>
+      </c>
+      <c r="L21" s="6">
+        <v>73.400000000000006</v>
+      </c>
+      <c r="M21" s="6">
+        <v>11.42</v>
+      </c>
+      <c r="N21" s="6">
+        <v>57.07</v>
+      </c>
+      <c r="O21" s="6">
+        <v>5.25</v>
+      </c>
+      <c r="P21" s="6">
+        <v>6.48</v>
+      </c>
+      <c r="Q21" s="6">
+        <v>3.45</v>
+      </c>
+      <c r="R21" s="6">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="6">
+        <v>7.59</v>
+      </c>
+      <c r="D22" s="6">
+        <v>489.79</v>
+      </c>
+      <c r="E22" s="6">
+        <v>40.21</v>
+      </c>
+      <c r="F22" s="6">
+        <v>769.65</v>
+      </c>
+      <c r="G22" s="6">
+        <v>6.76</v>
+      </c>
+      <c r="H22" s="6">
+        <v>335.92</v>
+      </c>
+      <c r="I22" s="6">
+        <v>327.11</v>
+      </c>
+      <c r="J22" s="6">
+        <v>374.13</v>
+      </c>
+      <c r="K22" s="6">
+        <v>25.98</v>
+      </c>
+      <c r="L22" s="6">
+        <v>74.52</v>
+      </c>
+      <c r="M22" s="6">
+        <v>11.55</v>
+      </c>
+      <c r="N22" s="6">
+        <v>57.07</v>
+      </c>
+      <c r="O22" s="6">
+        <v>5.3</v>
+      </c>
+      <c r="P22" s="6">
+        <v>6.28</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>3.3</v>
+      </c>
+      <c r="R22" s="6">
+        <v>3.21</v>
+      </c>
+    </row>
+    <row r="23" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="6">
+        <v>7.23</v>
+      </c>
+      <c r="D23" s="6">
+        <v>484.92</v>
+      </c>
+      <c r="E23" s="6">
+        <v>38.94</v>
+      </c>
+      <c r="F23" s="6">
+        <v>751.11</v>
+      </c>
+      <c r="G23" s="6">
+        <v>4.53</v>
+      </c>
+      <c r="H23" s="6">
+        <v>334.62</v>
+      </c>
+      <c r="I23" s="6">
+        <v>326.62</v>
+      </c>
+      <c r="J23" s="6">
+        <v>352</v>
+      </c>
+      <c r="K23" s="6">
+        <v>26.32</v>
+      </c>
+      <c r="L23" s="6">
+        <v>75.83</v>
+      </c>
+      <c r="M23" s="6">
+        <v>11.83</v>
+      </c>
+      <c r="N23" s="6">
+        <v>60.1</v>
+      </c>
+      <c r="O23" s="6">
+        <v>5.45</v>
+      </c>
+      <c r="P23" s="6">
+        <v>6.17</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>3.51</v>
+      </c>
+      <c r="R23" s="6">
+        <v>3.43</v>
+      </c>
+    </row>
+    <row r="24" spans="2:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="6">
+        <v>7.15</v>
+      </c>
+      <c r="D24" s="6">
+        <v>412.57</v>
+      </c>
+      <c r="E24" s="6">
+        <v>37.450000000000003</v>
+      </c>
+      <c r="F24" s="6">
+        <v>690.01</v>
+      </c>
+      <c r="G24" s="6">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="H24" s="6">
+        <v>328.9</v>
+      </c>
+      <c r="I24" s="6">
+        <v>316.94</v>
+      </c>
+      <c r="J24" s="6">
+        <v>346</v>
+      </c>
+      <c r="K24" s="6">
+        <v>25.77</v>
+      </c>
+      <c r="L24" s="6">
+        <v>72</v>
+      </c>
+      <c r="M24" s="6">
+        <v>11.11</v>
+      </c>
+      <c r="N24" s="6">
+        <v>55.48</v>
+      </c>
+      <c r="O24" s="6">
+        <v>5.15</v>
+      </c>
+      <c r="P24" s="6">
+        <v>6.59</v>
+      </c>
+      <c r="Q24" s="6">
+        <v>3.3</v>
+      </c>
+      <c r="R24" s="6">
+        <v>3.18</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C3:C24">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D24">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3:E24">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F24">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G24">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H24">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I24">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J24">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K24">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:L24">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:M24">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N3:N24">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O3:O24">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3:P24">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q3:Q24">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R3:R24">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>